<commit_message>
feat: add characters to compilation
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8BCD8D-7623-4EB7-9706-356EFE4D67A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571A8113-B985-4FDB-891B-88029CC11EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
     <sheet name="Locations" sheetId="2" r:id="rId2"/>
+    <sheet name="Characters" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="98">
   <si>
     <t>Name</t>
   </si>
@@ -328,6 +329,9 @@
   </si>
   <si>
     <t>Day of Disaster</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
 </sst>
 </file>
@@ -1972,4 +1976,85 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADEB2227-4206-4454-8691-07022EF9BF9A}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Thunderbirds compilation
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571A8113-B985-4FDB-891B-88029CC11EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BED69B-28F1-46C8-83E0-1758771B3D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
     <sheet name="Locations" sheetId="2" r:id="rId2"/>
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
+    <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="100">
   <si>
     <t>Name</t>
   </si>
@@ -332,6 +333,12 @@
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>Thunderbird 2</t>
+  </si>
+  <si>
+    <t>Thunderbird 5</t>
   </si>
 </sst>
 </file>
@@ -2057,4 +2064,49 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: fix typo in Rockquake!
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9256970-B2D1-4962-BF8E-4C238FD409C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B48026-E89E-4266-83F8-5F69E270A15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -180,9 +180,6 @@
     <t>Mole</t>
   </si>
   <si>
-    <t>Rockquake</t>
-  </si>
-  <si>
     <t>Australia</t>
   </si>
   <si>
@@ -340,6 +337,9 @@
   </si>
   <si>
     <t>Thunderbird 5</t>
+  </si>
+  <si>
+    <t>Rockquake!</t>
   </si>
 </sst>
 </file>
@@ -975,37 +975,37 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="B9">
         <v>10</v>
       </c>
       <c r="C9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
         <v>47</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>48</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="H9" t="s">
         <v>49</v>
       </c>
-      <c r="F9">
-        <v>2</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9">
+        <v>2</v>
+      </c>
+      <c r="K9" t="s">
         <v>50</v>
       </c>
-      <c r="I9">
-        <v>2</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="L9">
+        <v>2</v>
+      </c>
+      <c r="N9" t="s">
         <v>51</v>
-      </c>
-      <c r="L9">
-        <v>2</v>
-      </c>
-      <c r="N9" t="s">
-        <v>52</v>
       </c>
       <c r="O9" t="s">
         <v>21</v>
@@ -1013,16 +1013,16 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
         <v>42</v>
@@ -1031,7 +1031,7 @@
         <v>2</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I10">
         <v>2</v>
@@ -1046,36 +1046,36 @@
         <v>27</v>
       </c>
       <c r="O10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
         <v>17</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="H11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I11">
         <v>2</v>
       </c>
       <c r="J11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K11" t="s">
         <v>19</v>
@@ -1084,10 +1084,10 @@
         <v>3</v>
       </c>
       <c r="M11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O11" t="s">
         <v>21</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B12">
         <v>8</v>
@@ -1107,7 +1107,7 @@
         <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -1124,7 +1124,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B13">
         <v>7</v>
@@ -1133,7 +1133,7 @@
         <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
@@ -1151,12 +1151,12 @@
         <v>40</v>
       </c>
       <c r="N13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14">
         <v>11</v>
@@ -1165,10 +1165,10 @@
         <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F14">
         <v>3</v>
@@ -1186,7 +1186,7 @@
         <v>2</v>
       </c>
       <c r="N14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O14" t="s">
         <v>21</v>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B15">
         <v>11</v>
@@ -1212,7 +1212,7 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I15">
         <v>2</v>
@@ -1224,7 +1224,7 @@
         <v>2</v>
       </c>
       <c r="N15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O15" t="s">
         <v>21</v>
@@ -1232,19 +1232,19 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16">
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F16">
         <v>2</v>
@@ -1256,15 +1256,15 @@
         <v>2</v>
       </c>
       <c r="N16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17">
         <v>10</v>
@@ -1282,13 +1282,13 @@
         <v>3</v>
       </c>
       <c r="H17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I17">
         <v>2</v>
       </c>
       <c r="N17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O17" t="s">
         <v>21</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B18">
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
@@ -1314,7 +1314,7 @@
         <v>2</v>
       </c>
       <c r="H18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I18">
         <v>3</v>
@@ -1328,7 +1328,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -1340,7 +1340,7 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F19">
         <v>3</v>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20">
         <v>11</v>
@@ -1369,7 +1369,7 @@
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F20">
         <v>3</v>
@@ -1381,7 +1381,7 @@
         <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L20">
         <v>2</v>
@@ -1395,13 +1395,13 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B21">
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D21" t="s">
         <v>17</v>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="M21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N21" t="s">
         <v>27</v>
@@ -1436,31 +1436,31 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B22">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D22" t="s">
         <v>17</v>
       </c>
       <c r="E22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F22">
         <v>2</v>
       </c>
       <c r="H22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I22">
         <v>2</v>
       </c>
       <c r="N22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O22" t="s">
         <v>27</v>
@@ -1468,13 +1468,13 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23">
         <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
@@ -1486,7 +1486,7 @@
         <v>2</v>
       </c>
       <c r="H23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I23">
         <v>2</v>
@@ -1497,19 +1497,19 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D24" t="s">
         <v>17</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F24">
         <v>2</v>
@@ -1524,7 +1524,7 @@
         <v>40</v>
       </c>
       <c r="N24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O24" t="s">
         <v>34</v>
@@ -1532,7 +1532,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25">
         <v>8</v>
@@ -1561,7 +1561,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26">
         <v>8</v>
@@ -1570,16 +1570,16 @@
         <v>32</v>
       </c>
       <c r="D26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F26">
         <v>3</v>
       </c>
       <c r="H26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I26">
         <v>2</v>
@@ -1590,13 +1590,13 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D27" t="s">
         <v>37</v>
@@ -1608,24 +1608,24 @@
         <v>2</v>
       </c>
       <c r="H27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I27">
         <v>2</v>
       </c>
       <c r="J27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N27" t="s">
         <v>27</v>
       </c>
       <c r="O27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -1637,7 +1637,7 @@
         <v>24</v>
       </c>
       <c r="E28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F28">
         <v>3</v>
@@ -1652,7 +1652,7 @@
         <v>32</v>
       </c>
       <c r="N28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O28" t="s">
         <v>34</v>
@@ -1660,19 +1660,19 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B29">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F29">
         <v>2</v>
@@ -1684,27 +1684,27 @@
         <v>3</v>
       </c>
       <c r="J29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N29" t="s">
         <v>34</v>
       </c>
       <c r="O29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B30">
         <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E30" t="s">
         <v>18</v>
@@ -1719,7 +1719,7 @@
         <v>2</v>
       </c>
       <c r="J30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N30" t="s">
         <v>21</v>
@@ -1727,7 +1727,7 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B31">
         <v>7</v>
@@ -1751,7 +1751,7 @@
         <v>2</v>
       </c>
       <c r="J31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N31" t="s">
         <v>27</v>
@@ -1759,13 +1759,13 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B32">
         <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
@@ -1783,12 +1783,12 @@
         <v>1</v>
       </c>
       <c r="N32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B33">
         <v>7</v>
@@ -1800,18 +1800,18 @@
         <v>24</v>
       </c>
       <c r="E33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F33">
         <v>3</v>
       </c>
       <c r="N33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B34">
         <v>9</v>
@@ -1838,36 +1838,36 @@
         <v>34</v>
       </c>
       <c r="O34" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B35">
         <v>8</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E35" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="H35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I35">
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L35">
         <v>2</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -1918,7 +1918,7 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -1928,42 +1928,42 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -1973,7 +1973,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
@@ -1999,15 +1999,15 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -2015,7 +2015,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
@@ -2048,7 +2048,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
@@ -2084,7 +2084,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -2099,7 +2099,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -2139,27 +2139,27 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -2169,7 +2169,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add fab/event cards to Excel
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF6FAD9-600A-4D02-ADB0-7F9607AA552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32ED6F80-A778-4421-84C1-C61C00DEFB2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
-    <sheet name="Map Edges" sheetId="7" r:id="rId6"/>
+    <sheet name="FAB Cards" sheetId="6" r:id="rId6"/>
+    <sheet name="Event Cards" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="130">
   <si>
     <t>Name</t>
   </si>
@@ -343,19 +344,94 @@
     <t>Rockquake!</t>
   </si>
   <si>
-    <t>Domain</t>
-  </si>
-  <si>
-    <t>Earth</t>
-  </si>
-  <si>
-    <t>Top Speed</t>
-  </si>
-  <si>
-    <t>Edge 1</t>
-  </si>
-  <si>
-    <t>Edge 2</t>
+    <t>The Hood Interferes</t>
+  </si>
+  <si>
+    <t>Explosion on Tracy Island</t>
+  </si>
+  <si>
+    <t>Pod Hydraulics Sabotaged</t>
+  </si>
+  <si>
+    <t>Attack of the Zombites</t>
+  </si>
+  <si>
+    <t>Accidental Injury</t>
+  </si>
+  <si>
+    <t>Rocket Malfunction</t>
+  </si>
+  <si>
+    <t>Kyrano… Kyrano!!</t>
+  </si>
+  <si>
+    <t>Emergency Comms Interrupted</t>
+  </si>
+  <si>
+    <t>The Hood's Hynoptic Eyes</t>
+  </si>
+  <si>
+    <t>USN Sentinel Missile Strike</t>
+  </si>
+  <si>
+    <t>Master of Disguise</t>
+  </si>
+  <si>
+    <t>Icelandic Volcano Eruption</t>
+  </si>
+  <si>
+    <t>Underwater Sealing Unit</t>
+  </si>
+  <si>
+    <t>Holiday in Bonga Bonga</t>
+  </si>
+  <si>
+    <t>Mobile Command Unit</t>
+  </si>
+  <si>
+    <t>Astronaut Spacewalk</t>
+  </si>
+  <si>
+    <t>Grandma's Cooking</t>
+  </si>
+  <si>
+    <t>Experimental Fuel</t>
+  </si>
+  <si>
+    <t>Air Sea Rescue Centre</t>
+  </si>
+  <si>
+    <t>Help from Braman</t>
+  </si>
+  <si>
+    <t>Powder Compact Radio</t>
+  </si>
+  <si>
+    <t>Automatic Camera Detector</t>
+  </si>
+  <si>
+    <t>Tracy Brothers' Portraits</t>
+  </si>
+  <si>
+    <t>Agent-47 Jeremiah Tuttle</t>
+  </si>
+  <si>
+    <t>FAB 1 Hydrofoils</t>
+  </si>
+  <si>
+    <t>Remote Control Hover Camera</t>
+  </si>
+  <si>
+    <t>Personal Hoverjet</t>
+  </si>
+  <si>
+    <t>Sir Jeremy Hodge</t>
+  </si>
+  <si>
+    <t>Long-Range Walkie Talkies</t>
+  </si>
+  <si>
+    <t>Jeff's Orders</t>
   </si>
 </sst>
 </file>
@@ -1899,159 +1975,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8390046B-9FE3-48A8-9F65-5552D9E8BDF3}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
-      <c r="B3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
-      <c r="B8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
-      <c r="B9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>67</v>
       </c>
-      <c r="B10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>88</v>
       </c>
-      <c r="B11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>46</v>
       </c>
-      <c r="B12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>76</v>
       </c>
-      <c r="B14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>91</v>
       </c>
-      <c r="B15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>57</v>
       </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>29</v>
       </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>72</v>
       </c>
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
-      </c>
-      <c r="B19" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2142,84 +2161,42 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
-      <c r="B3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>98</v>
       </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2293,338 +2270,178 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E42479-0211-470A-B268-566711210746}">
-  <dimension ref="A1:C30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0DC219-ECA6-4590-958F-6BDC2A6EF2E8}">
+  <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA6DCDF-51E7-4440-B5D3-A355F5D584CF}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>103</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>104</v>
       </c>
-      <c r="C1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>86</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B25" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>91</v>
-      </c>
-      <c r="B27" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>73</v>
-      </c>
-      <c r="B28" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" t="s">
-        <v>72</v>
-      </c>
-      <c r="C29" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" t="s">
-        <v>17</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: spelling error in hypnotic
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32ED6F80-A778-4421-84C1-C61C00DEFB2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4587A66-2021-4653-A42E-52A4359C520F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -368,9 +368,6 @@
     <t>Emergency Comms Interrupted</t>
   </si>
   <si>
-    <t>The Hood's Hynoptic Eyes</t>
-  </si>
-  <si>
     <t>USN Sentinel Missile Strike</t>
   </si>
   <si>
@@ -432,6 +429,9 @@
   </si>
   <si>
     <t>Jeff's Orders</t>
+  </si>
+  <si>
+    <t>The Hood's Hypnotic Eyes</t>
   </si>
 </sst>
 </file>
@@ -2281,92 +2281,92 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2426,22 +2426,22 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update reference source data
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B48026-E89E-4266-83F8-5F69E270A15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF6FAD9-600A-4D02-ADB0-7F9607AA552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
+    <sheet name="Map Edges" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="105">
   <si>
     <t>Name</t>
   </si>
@@ -340,6 +341,21 @@
   </si>
   <si>
     <t>Rockquake!</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>Top Speed</t>
+  </si>
+  <si>
+    <t>Edge 1</t>
+  </si>
+  <si>
+    <t>Edge 2</t>
   </si>
 </sst>
 </file>
@@ -1883,102 +1899,159 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8390046B-9FE3-48A8-9F65-5552D9E8BDF3}">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2069,42 +2142,84 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2175,4 +2290,344 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E42479-0211-470A-B268-566711210746}">
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
tests: resolve merge issues post rebase
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4587A66-2021-4653-A42E-52A4359C520F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573B8EBE-2E58-4165-9FB5-7215CAD8CAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
-    <sheet name="FAB Cards" sheetId="6" r:id="rId6"/>
-    <sheet name="Event Cards" sheetId="7" r:id="rId7"/>
+    <sheet name="Map Edges" sheetId="8" r:id="rId6"/>
+    <sheet name="FAB Cards" sheetId="6" r:id="rId7"/>
+    <sheet name="Event Cards" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="135">
   <si>
     <t>Name</t>
   </si>
@@ -432,6 +433,21 @@
   </si>
   <si>
     <t>The Hood's Hypnotic Eyes</t>
+  </si>
+  <si>
+    <t>Edge 1</t>
+  </si>
+  <si>
+    <t>Edge 2</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>Top Speed</t>
   </si>
 </sst>
 </file>
@@ -467,7 +483,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1975,102 +1993,159 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8390046B-9FE3-48A8-9F65-5552D9E8BDF3}">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B1" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B3" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B4" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B5" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B6" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B7" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B8" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B9" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B10" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B11" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B12" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B13" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B15" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B16" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B17" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="B18" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2161,42 +2236,84 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B2" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B3" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B5" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2270,6 +2387,346 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B37DDD8-053B-497B-A0FD-20F208B606C5}">
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0DC219-ECA6-4590-958F-6BDC2A6EF2E8}">
   <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2374,7 +2831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA6DCDF-51E7-4440-B5D3-A355F5D584CF}">
   <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
chore: intialise F.A.B. in Excel source to align with presentation standards
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573B8EBE-2E58-4165-9FB5-7215CAD8CAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F7A40A-3752-4C06-83AB-BAFE40D224DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
     <sheet name="Map Edges" sheetId="8" r:id="rId6"/>
-    <sheet name="FAB Cards" sheetId="6" r:id="rId7"/>
+    <sheet name="F.A.B. Cards" sheetId="6" r:id="rId7"/>
     <sheet name="Event Cards" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -483,9 +483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1997,154 +1995,154 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>67</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>88</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" t="s">
         <v>76</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>91</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="A18" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2240,79 +2238,79 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>132</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>98</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="B7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rescue card modifiers (#64)
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF6FAD9-600A-4D02-ADB0-7F9607AA552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F7A40A-3752-4C06-83AB-BAFE40D224DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,9 @@
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
-    <sheet name="Map Edges" sheetId="7" r:id="rId6"/>
+    <sheet name="Map Edges" sheetId="8" r:id="rId6"/>
+    <sheet name="F.A.B. Cards" sheetId="6" r:id="rId7"/>
+    <sheet name="Event Cards" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="135">
   <si>
     <t>Name</t>
   </si>
@@ -343,6 +345,102 @@
     <t>Rockquake!</t>
   </si>
   <si>
+    <t>The Hood Interferes</t>
+  </si>
+  <si>
+    <t>Explosion on Tracy Island</t>
+  </si>
+  <si>
+    <t>Pod Hydraulics Sabotaged</t>
+  </si>
+  <si>
+    <t>Attack of the Zombites</t>
+  </si>
+  <si>
+    <t>Accidental Injury</t>
+  </si>
+  <si>
+    <t>Rocket Malfunction</t>
+  </si>
+  <si>
+    <t>Kyrano… Kyrano!!</t>
+  </si>
+  <si>
+    <t>Emergency Comms Interrupted</t>
+  </si>
+  <si>
+    <t>USN Sentinel Missile Strike</t>
+  </si>
+  <si>
+    <t>Master of Disguise</t>
+  </si>
+  <si>
+    <t>Icelandic Volcano Eruption</t>
+  </si>
+  <si>
+    <t>Underwater Sealing Unit</t>
+  </si>
+  <si>
+    <t>Holiday in Bonga Bonga</t>
+  </si>
+  <si>
+    <t>Mobile Command Unit</t>
+  </si>
+  <si>
+    <t>Astronaut Spacewalk</t>
+  </si>
+  <si>
+    <t>Grandma's Cooking</t>
+  </si>
+  <si>
+    <t>Experimental Fuel</t>
+  </si>
+  <si>
+    <t>Air Sea Rescue Centre</t>
+  </si>
+  <si>
+    <t>Help from Braman</t>
+  </si>
+  <si>
+    <t>Powder Compact Radio</t>
+  </si>
+  <si>
+    <t>Automatic Camera Detector</t>
+  </si>
+  <si>
+    <t>Tracy Brothers' Portraits</t>
+  </si>
+  <si>
+    <t>Agent-47 Jeremiah Tuttle</t>
+  </si>
+  <si>
+    <t>FAB 1 Hydrofoils</t>
+  </si>
+  <si>
+    <t>Remote Control Hover Camera</t>
+  </si>
+  <si>
+    <t>Personal Hoverjet</t>
+  </si>
+  <si>
+    <t>Sir Jeremy Hodge</t>
+  </si>
+  <si>
+    <t>Long-Range Walkie Talkies</t>
+  </si>
+  <si>
+    <t>Jeff's Orders</t>
+  </si>
+  <si>
+    <t>The Hood's Hypnotic Eyes</t>
+  </si>
+  <si>
+    <t>Edge 1</t>
+  </si>
+  <si>
+    <t>Edge 2</t>
+  </si>
+  <si>
     <t>Domain</t>
   </si>
   <si>
@@ -350,12 +448,6 @@
   </si>
   <si>
     <t>Top Speed</t>
-  </si>
-  <si>
-    <t>Edge 1</t>
-  </si>
-  <si>
-    <t>Edge 2</t>
   </si>
 </sst>
 </file>
@@ -1907,7 +1999,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1915,7 +2007,7 @@
         <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1923,7 +2015,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1931,7 +2023,7 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1939,7 +2031,7 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1947,7 +2039,7 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1955,7 +2047,7 @@
         <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1963,7 +2055,7 @@
         <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1971,7 +2063,7 @@
         <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1979,7 +2071,7 @@
         <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1987,7 +2079,7 @@
         <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1995,7 +2087,7 @@
         <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2150,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2161,7 +2253,7 @@
         <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C2">
         <v>3</v>
@@ -2172,7 +2264,7 @@
         <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -2194,7 +2286,7 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2216,7 +2308,7 @@
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -2293,19 +2385,19 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E42479-0211-470A-B268-566711210746}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B37DDD8-053B-497B-A0FD-20F208B606C5}">
   <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2316,7 +2408,7 @@
         <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2327,7 +2419,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2338,7 +2430,7 @@
         <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2349,7 +2441,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2360,7 +2452,7 @@
         <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2371,7 +2463,7 @@
         <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2382,7 +2474,7 @@
         <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2393,7 +2485,7 @@
         <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2404,7 +2496,7 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2415,7 +2507,7 @@
         <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2426,7 +2518,7 @@
         <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2437,7 +2529,7 @@
         <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2448,7 +2540,7 @@
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2459,7 +2551,7 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2470,7 +2562,7 @@
         <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2481,7 +2573,7 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2492,7 +2584,7 @@
         <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -2503,7 +2595,7 @@
         <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -2514,7 +2606,7 @@
         <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2525,7 +2617,7 @@
         <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2536,7 +2628,7 @@
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2547,7 +2639,7 @@
         <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2625,6 +2717,186 @@
       </c>
       <c r="C30" t="s">
         <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0DC219-ECA6-4590-958F-6BDC2A6EF2E8}">
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA6DCDF-51E7-4440-B5D3-A355F5D584CF}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>